<commit_message>
fix: v8 Tab3 미코딩 11건 코딩 완료 (#11,#47,#49-57)
- I (Include) 6건: #49(TAM/PE/EE/BI/SE), #51(PLS-SEM/PE/EE/FC/ATT),
  #53(SEM/FC/PE/ATT), #55(PLS-SEM/TRU/PE), #56(UTAUT2/SEM-ANN),
  #57(AIDUA/SEM)
- X (Exclude) 5건: #11(E-FT6/DOI오류), #47(E-FT1/상관없음),
  #50(E-FT2/TPACK), #52(E-FT2/챗봇효과), #54(E-FT2/FLCA≠AI불안)
- 하단 고아 DOI 행(138-152) 정리

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/human_review_sheet_v8.xlsx
+++ b/data/templates/human_review_sheet_v8.xlsx
@@ -28660,9 +28660,21 @@
           <t>include+uncertain</t>
         </is>
       </c>
-      <c r="J13" s="27" t="n"/>
-      <c r="K13" s="27" t="n"/>
-      <c r="L13" s="28" t="n"/>
+      <c r="J13" s="27" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K13" s="27" t="inlineStr">
+        <is>
+          <t>E-FT6</t>
+        </is>
+      </c>
+      <c r="L13" s="28" t="inlineStr">
+        <is>
+          <t>DOI 오류(COVID 백신 논문으로 연결), 원문 확인 불가</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="36" t="n">
@@ -30540,9 +30552,21 @@
           <t>uncertain+include</t>
         </is>
       </c>
-      <c r="J49" s="27" t="n"/>
-      <c r="K49" s="27" t="n"/>
-      <c r="L49" s="28" t="n"/>
+      <c r="J49" s="27" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K49" s="27" t="inlineStr">
+        <is>
+          <t>E-FT1</t>
+        </is>
+      </c>
+      <c r="L49" s="28" t="inlineStr">
+        <is>
+          <t>기술적 설문조사(screening method), 상관행렬/회귀계수 없음</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="28" customHeight="1">
       <c r="A50" s="36" t="n">
@@ -30636,9 +30660,17 @@
           <t>include+uncertain</t>
         </is>
       </c>
-      <c r="J51" s="27" t="n"/>
+      <c r="J51" s="27" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="K51" s="27" t="n"/>
-      <c r="L51" s="28" t="n"/>
+      <c r="L51" s="28" t="inlineStr">
+        <is>
+          <t>TAM 확장, PE/EE/BI/SE 포함, humanoid robot 수용, 508명, SPSS</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="28" customHeight="1">
       <c r="A52" s="36" t="n">
@@ -30682,9 +30714,21 @@
           <t>include+uncertain</t>
         </is>
       </c>
-      <c r="J52" s="27" t="n"/>
-      <c r="K52" s="27" t="n"/>
-      <c r="L52" s="28" t="n"/>
+      <c r="J52" s="27" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K52" s="27" t="inlineStr">
+        <is>
+          <t>E-FT2</t>
+        </is>
+      </c>
+      <c r="L52" s="28" t="inlineStr">
+        <is>
+          <t>TPACK 프레임워크, 수용 construct 아님 (art+AI 교육모형 개발)</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="28" customHeight="1">
       <c r="A53" s="36" t="n">
@@ -30728,9 +30772,17 @@
           <t>include+uncertain</t>
         </is>
       </c>
-      <c r="J53" s="27" t="n"/>
+      <c r="J53" s="27" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="K53" s="27" t="n"/>
-      <c r="L53" s="28" t="n"/>
+      <c r="L53" s="28" t="inlineStr">
+        <is>
+          <t>PLS-SEM, PE/EE/FC/ATT 포함, 아시아 7개국 교수 대상</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="28" customHeight="1">
       <c r="A54" s="36" t="n">
@@ -30774,9 +30826,21 @@
           <t>include+uncertain</t>
         </is>
       </c>
-      <c r="J54" s="27" t="n"/>
-      <c r="K54" s="27" t="n"/>
-      <c r="L54" s="28" t="n"/>
+      <c r="J54" s="27" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K54" s="27" t="inlineStr">
+        <is>
+          <t>E-FT2</t>
+        </is>
+      </c>
+      <c r="L54" s="28" t="inlineStr">
+        <is>
+          <t>챗봇 효과 연구(self-efficacy/engagement), 수용 construct 2개 미만</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="28" customHeight="1">
       <c r="A55" s="36" t="n">
@@ -30820,9 +30884,17 @@
           <t>include+uncertain</t>
         </is>
       </c>
-      <c r="J55" s="27" t="n"/>
+      <c r="J55" s="27" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="K55" s="27" t="n"/>
-      <c r="L55" s="28" t="n"/>
+      <c r="L55" s="28" t="inlineStr">
+        <is>
+          <t>SEM, FC/PE/ATT 포함, 720명, AI 통합 태도</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="36" t="n">
@@ -30866,9 +30938,21 @@
           <t>include+uncertain</t>
         </is>
       </c>
-      <c r="J56" s="27" t="n"/>
-      <c r="K56" s="27" t="n"/>
-      <c r="L56" s="28" t="n"/>
+      <c r="J56" s="27" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K56" s="27" t="inlineStr">
+        <is>
+          <t>E-FT2</t>
+        </is>
+      </c>
+      <c r="L56" s="28" t="inlineStr">
+        <is>
+          <t>GenAI ATT만 해당, FLCA는 AI 불안 아님, 수용 construct 2개 미만</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="36" t="n">
@@ -30912,9 +30996,17 @@
           <t>include+uncertain</t>
         </is>
       </c>
-      <c r="J57" s="27" t="n"/>
+      <c r="J57" s="27" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="K57" s="27" t="n"/>
-      <c r="L57" s="28" t="n"/>
+      <c r="L57" s="28" t="inlineStr">
+        <is>
+          <t>PLS-SEM, TRU/PE 포함, 간호교육, 팔레스타인</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="36" t="n">
@@ -30958,9 +31050,17 @@
           <t>uncertain+include</t>
         </is>
       </c>
-      <c r="J58" s="27" t="n"/>
+      <c r="J58" s="27" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="K58" s="27" t="n"/>
-      <c r="L58" s="28" t="n"/>
+      <c r="L58" s="28" t="inlineStr">
+        <is>
+          <t>UTAUT2 확장, PE/EE/SI/FC/BI/UB 포함, SEM-ANN 하이브리드, 가나</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="36" t="n">
@@ -31004,9 +31104,17 @@
           <t>uncertain+include</t>
         </is>
       </c>
-      <c r="J59" s="27" t="n"/>
+      <c r="J59" s="27" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="K59" s="27" t="n"/>
-      <c r="L59" s="28" t="n"/>
+      <c r="L59" s="28" t="inlineStr">
+        <is>
+          <t>AIDUA 모델, SEM, 에콰도르 220명, cognition-motivation-emotion 프레임워크</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="36" t="n">
@@ -34609,11 +34717,7 @@
       <c r="B138" s="36" t="n"/>
       <c r="C138" s="37" t="n"/>
       <c r="D138" s="36" t="n"/>
-      <c r="E138" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1080/02188791.2025.2564138</t>
-        </is>
-      </c>
+      <c r="E138" s="38" t="n"/>
       <c r="F138" s="36" t="n"/>
       <c r="G138" s="36" t="n"/>
       <c r="H138" s="37" t="n"/>
@@ -34627,11 +34731,7 @@
       <c r="B139" s="36" t="n"/>
       <c r="C139" s="37" t="n"/>
       <c r="D139" s="36" t="n"/>
-      <c r="E139" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1080/10494820.2025.2596061</t>
-        </is>
-      </c>
+      <c r="E139" s="38" t="n"/>
       <c r="F139" s="36" t="n"/>
       <c r="G139" s="36" t="n"/>
       <c r="H139" s="37" t="n"/>
@@ -34645,11 +34745,7 @@
       <c r="B140" s="36" t="n"/>
       <c r="C140" s="37" t="n"/>
       <c r="D140" s="36" t="n"/>
-      <c r="E140" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.22521/edupij.2025.17.309</t>
-        </is>
-      </c>
+      <c r="E140" s="38" t="n"/>
       <c r="F140" s="36" t="n"/>
       <c r="G140" s="36" t="n"/>
       <c r="H140" s="37" t="n"/>
@@ -34663,11 +34759,7 @@
       <c r="B141" s="36" t="n"/>
       <c r="C141" s="37" t="n"/>
       <c r="D141" s="36" t="n"/>
-      <c r="E141" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1080/02188791.2025.2577334</t>
-        </is>
-      </c>
+      <c r="E141" s="38" t="n"/>
       <c r="F141" s="36" t="n"/>
       <c r="G141" s="36" t="n"/>
       <c r="H141" s="37" t="n"/>
@@ -34681,11 +34773,7 @@
       <c r="B142" s="36" t="n"/>
       <c r="C142" s="37" t="n"/>
       <c r="D142" s="36" t="n"/>
-      <c r="E142" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1080/10528008.2023.2300139</t>
-        </is>
-      </c>
+      <c r="E142" s="38" t="n"/>
       <c r="F142" s="36" t="n"/>
       <c r="G142" s="36" t="n"/>
       <c r="H142" s="37" t="n"/>
@@ -34699,11 +34787,7 @@
       <c r="B143" s="36" t="n"/>
       <c r="C143" s="37" t="n"/>
       <c r="D143" s="36" t="n"/>
-      <c r="E143" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.3390/su17125609</t>
-        </is>
-      </c>
+      <c r="E143" s="38" t="n"/>
       <c r="F143" s="36" t="n"/>
       <c r="G143" s="36" t="n"/>
       <c r="H143" s="37" t="n"/>
@@ -34717,11 +34801,7 @@
       <c r="B144" s="36" t="n"/>
       <c r="C144" s="37" t="n"/>
       <c r="D144" s="36" t="n"/>
-      <c r="E144" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1145/3611313</t>
-        </is>
-      </c>
+      <c r="E144" s="38" t="n"/>
       <c r="F144" s="36" t="n"/>
       <c r="G144" s="36" t="n"/>
       <c r="H144" s="37" t="n"/>
@@ -34735,11 +34815,7 @@
       <c r="B145" s="36" t="n"/>
       <c r="C145" s="37" t="n"/>
       <c r="D145" s="36" t="n"/>
-      <c r="E145" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1108/JARHE-03-2024-0126</t>
-        </is>
-      </c>
+      <c r="E145" s="38" t="n"/>
       <c r="F145" s="36" t="n"/>
       <c r="G145" s="36" t="n"/>
       <c r="H145" s="37" t="n"/>
@@ -34753,11 +34829,7 @@
       <c r="B146" s="36" t="n"/>
       <c r="C146" s="37" t="n"/>
       <c r="D146" s="36" t="n"/>
-      <c r="E146" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1108/JARHE-04-2025-0256</t>
-        </is>
-      </c>
+      <c r="E146" s="38" t="n"/>
       <c r="F146" s="36" t="n"/>
       <c r="G146" s="36" t="n"/>
       <c r="H146" s="37" t="n"/>
@@ -34771,11 +34843,7 @@
       <c r="B147" s="36" t="n"/>
       <c r="C147" s="37" t="n"/>
       <c r="D147" s="36" t="n"/>
-      <c r="E147" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.ijedudev.2025.103434</t>
-        </is>
-      </c>
+      <c r="E147" s="38" t="n"/>
       <c r="F147" s="36" t="n"/>
       <c r="G147" s="36" t="n"/>
       <c r="H147" s="37" t="n"/>
@@ -34789,11 +34857,7 @@
       <c r="B148" s="36" t="n"/>
       <c r="C148" s="37" t="n"/>
       <c r="D148" s="36" t="n"/>
-      <c r="E148" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.3389/fpsyg.2024.1447680</t>
-        </is>
-      </c>
+      <c r="E148" s="38" t="n"/>
       <c r="F148" s="36" t="n"/>
       <c r="G148" s="36" t="n"/>
       <c r="H148" s="37" t="n"/>
@@ -34807,11 +34871,7 @@
       <c r="B149" s="36" t="n"/>
       <c r="C149" s="37" t="n"/>
       <c r="D149" s="36" t="n"/>
-      <c r="E149" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.ijer.2025.102636</t>
-        </is>
-      </c>
+      <c r="E149" s="38" t="n"/>
       <c r="F149" s="36" t="n"/>
       <c r="G149" s="36" t="n"/>
       <c r="H149" s="37" t="n"/>
@@ -34825,11 +34885,7 @@
       <c r="B150" s="36" t="n"/>
       <c r="C150" s="37" t="n"/>
       <c r="D150" s="36" t="n"/>
-      <c r="E150" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1155/hbe2/1518987</t>
-        </is>
-      </c>
+      <c r="E150" s="38" t="n"/>
       <c r="F150" s="36" t="n"/>
       <c r="G150" s="36" t="n"/>
       <c r="H150" s="37" t="n"/>
@@ -34843,11 +34899,7 @@
       <c r="B151" s="36" t="n"/>
       <c r="C151" s="37" t="n"/>
       <c r="D151" s="36" t="n"/>
-      <c r="E151" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.23925/2179-3565.2025v16i3p13-25</t>
-        </is>
-      </c>
+      <c r="E151" s="38" t="n"/>
       <c r="F151" s="36" t="n"/>
       <c r="G151" s="36" t="n"/>
       <c r="H151" s="37" t="n"/>
@@ -34861,11 +34913,7 @@
       <c r="B152" s="36" t="n"/>
       <c r="C152" s="37" t="n"/>
       <c r="D152" s="36" t="n"/>
-      <c r="E152" s="38" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.3389/fpsyg.2024.1466566</t>
-        </is>
-      </c>
+      <c r="E152" s="38" t="n"/>
       <c r="F152" s="36" t="n"/>
       <c r="G152" s="36" t="n"/>
       <c r="H152" s="37" t="n"/>
@@ -35024,21 +35072,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E135" r:id="rId133"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" r:id="rId134"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E137" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E138" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E139" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E141" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E142" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E143" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E144" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E145" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E146" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E147" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E148" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E149" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E150" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E151" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E152" r:id="rId150"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -36082,7 +36115,6 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
@@ -36131,7 +36163,6 @@
         </is>
       </c>
     </row>
-    <row r="72"/>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
@@ -36139,7 +36170,6 @@
         </is>
       </c>
     </row>
-    <row r="74"/>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
@@ -36200,7 +36230,6 @@
         </is>
       </c>
     </row>
-    <row r="80"/>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>

</xml_diff>